<commit_message>
Movilización: well cost 600k (SierraCol range 550–650k); campaign-level savings framing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Simulador_Movilizacion_GRS110.xlsx
+++ b/movilizacion/entregables/Simulador_Movilizacion_GRS110.xlsx
@@ -132,7 +132,7 @@
     <t xml:space="preserve">Tarifas.xlsx · E7. Se cancela con el WO; ver Pendientes</t>
   </si>
   <si>
-    <t xml:space="preserve">Costo de un pozo en LCI, solo perforación (USD) · SierraCol: 500–600 k</t>
+    <t xml:space="preserve">Costo de un pozo en LCI, solo perforación (USD) · SierraCol: 550–650 k</t>
   </si>
   <si>
     <t xml:space="preserve">Adicionales sobre Lump Sum</t>
@@ -2019,7 +2019,7 @@
     <t xml:space="preserve">Ahorro campaña (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">% del costo de un pozo (550 k)</t>
+    <t xml:space="preserve">% del costo de un pozo (600 k)</t>
   </si>
   <si>
     <t xml:space="preserve">Horas extra de taladro por movilización que lo anulan</t>
@@ -3445,7 +3445,7 @@
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
       <c r="N11" s="15" t="n">
-        <v>550000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="M84" s="27" t="n">
         <f aca="false">IF($N$11=0,0,L84/$N$11)</f>
-        <v>0.0078486550789751</v>
+        <v>0.00719460048906051</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="M85" s="27" t="n">
         <f aca="false">IF($N$11=0,0,L85/$N$11)</f>
-        <v>-0.0235772316181116</v>
+        <v>-0.0216124623166023</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4979,7 +4979,7 @@
       </c>
       <c r="M86" s="27" t="n">
         <f aca="false">IF($N$11=0,0,L86/$N$11)</f>
-        <v>-0.0235772316181116</v>
+        <v>-0.0216124623166023</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="M87" s="27" t="n">
         <f aca="false">IF($N$11=0,0,L87/$N$11)</f>
-        <v>0.0264651375219375</v>
+        <v>0.0242597093951094</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22206,7 +22206,7 @@
         <v>4316.76029343632</v>
       </c>
       <c r="F18" s="51" t="n">
-        <v>0.00784865507897512</v>
+        <v>0.00719460048906053</v>
       </c>
       <c r="G18" s="52" t="n">
         <v>2.96480789384362</v>
@@ -22238,7 +22238,7 @@
         <v>14555.8256370657</v>
       </c>
       <c r="F19" s="51" t="n">
-        <v>0.0264651375219376</v>
+        <v>0.0242597093951094</v>
       </c>
       <c r="G19" s="52" t="n">
         <v>9.99713299249015</v>
@@ -22270,7 +22270,7 @@
         <v>14979.3966872587</v>
       </c>
       <c r="F20" s="51" t="n">
-        <v>0.0272352667041067</v>
+        <v>0.0249656611454312</v>
       </c>
       <c r="G20" s="52" t="n">
         <v>10.288047175315</v>
@@ -22302,7 +22302,7 @@
         <v>16777.2542857143</v>
       </c>
       <c r="F21" s="51" t="n">
-        <v>0.0305040987012988</v>
+        <v>0.0279620904761905</v>
       </c>
       <c r="G21" s="52" t="n">
         <v>11.5228394819467</v>

</xml_diff>